<commit_message>
Make the scripts runnable from a fresh clone; add README
- Resolve paths relative to src/ instead of a hard-coded local folder:
  inputs in src/data/, results in src/output/ (already git-ignored)
- Remove the hard-coded ffmpeg path (ffmpeg is taken from PATH)
- Move POM.json to src/data/ and point case58-60 to it
- Add the FFCM-2 formaldehyde sub-model used by counterflow_SS.py
- Add the CH2O entry to polymer_evaporation.xlsx (needed by case58-60)
- Add README, requirements.txt, and ignore __pycache__/
</commit_message>
<xml_diff>
--- a/src/data/polymer_evaporation.xlsx
+++ b/src/data/polymer_evaporation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\14407\Documents\GitHub\Polymer\src\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\14407\AppData\Local\Temp\claude\D--OneDrive-DocumentAll-CV\69b58f8b-9797-427a-ba88-e48801a9fe8b\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81030FAC-8049-41CD-AB2B-C7E79AC98412}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A7270F3-BD3B-49B3-9D92-1D9488F4B3A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{E834531C-69FF-4871-B001-224ACE17D463}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{E834531C-69FF-4871-B001-224ACE17D463}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>Name</t>
   </si>
@@ -126,6 +126,9 @@
   </si>
   <si>
     <t>D</t>
+  </si>
+  <si>
+    <t>CH2O</t>
   </si>
 </sst>
 </file>
@@ -509,7 +512,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90EAB0A0-C382-4244-AE47-393084D9E6A6}">
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -891,6 +894,18 @@
         <v>0.14000000000000001</v>
       </c>
     </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="A12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H12">
+        <v>30</v>
+      </c>
+      <c r="I12">
+        <f>H12*0.001</f>
+        <v>0.03</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>